<commit_message>
Atualizando banco de dados: BASE_HISTORICA_AGENDAMENTOS.xlsx
</commit_message>
<xml_diff>
--- a/BASE_HISTORICA_AGENDAMENTOS.xlsx
+++ b/BASE_HISTORICA_AGENDAMENTOS.xlsx
@@ -415,7 +415,15 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Servico</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>